<commit_message>
updated the GAC-PAQ pages
</commit_message>
<xml_diff>
--- a/GACPAQ pages.xlsx
+++ b/GACPAQ pages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doncastillo/Code/gacpaq/gacpaq-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56686A86-3F82-794B-9BE7-36B735D17A6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76F6DB1-ED31-AF4B-BE57-88CA974F4891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20060" yWindow="-20860" windowWidth="38400" windowHeight="21100" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
+    <workbookView xWindow="19720" yWindow="-21100" windowWidth="38400" windowHeight="21100" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="969" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="422">
   <si>
     <t>Page Number</t>
   </si>
@@ -8007,7 +8007,9 @@
       <c r="F5" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="G5" s="55"/>
+      <c r="G5" s="56" t="s">
+        <v>415</v>
+      </c>
       <c r="H5" s="53" t="s">
         <v>337</v>
       </c>

</xml_diff>

<commit_message>
updated app to v3.8.4
</commit_message>
<xml_diff>
--- a/GACPAQ pages.xlsx
+++ b/GACPAQ pages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doncastillo/Code/gacpaq/gacpaq-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76F6DB1-ED31-AF4B-BE57-88CA974F4891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC74EE7C-8643-E448-9E10-69FBF77E6FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19720" yWindow="-21100" windowWidth="38400" windowHeight="21100" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
+    <workbookView xWindow="18060" yWindow="-20240" windowWidth="38400" windowHeight="21100" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="423">
   <si>
     <t>Page Number</t>
   </si>
@@ -2881,6 +2881,9 @@
   </si>
   <si>
     <t>on-going (12)</t>
+  </si>
+  <si>
+    <t>on-going (13)</t>
   </si>
 </sst>
 </file>
@@ -8249,7 +8252,9 @@
       <c r="J9" s="56" t="s">
         <v>419</v>
       </c>
-      <c r="K9" s="55"/>
+      <c r="K9" s="54" t="s">
+        <v>422</v>
+      </c>
       <c r="L9" s="40" t="s">
         <v>416</v>
       </c>
@@ -8305,7 +8310,9 @@
       <c r="J10" s="56" t="s">
         <v>419</v>
       </c>
-      <c r="K10" s="55"/>
+      <c r="K10" s="54" t="s">
+        <v>422</v>
+      </c>
       <c r="L10" s="40" t="s">
         <v>281</v>
       </c>
@@ -8361,7 +8368,9 @@
       <c r="J11" s="56" t="s">
         <v>419</v>
       </c>
-      <c r="K11" s="55"/>
+      <c r="K11" s="54" t="s">
+        <v>422</v>
+      </c>
       <c r="L11" s="40" t="s">
         <v>283</v>
       </c>

</xml_diff>

<commit_message>
updated the main study languages
</commit_message>
<xml_diff>
--- a/GACPAQ pages.xlsx
+++ b/GACPAQ pages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doncastillo/Code/gacpaq/gacpaq-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC74EE7C-8643-E448-9E10-69FBF77E6FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75C33FF3-592B-564B-A718-8AD9A7614087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18060" yWindow="-20240" windowWidth="38400" windowHeight="21100" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
+    <workbookView xWindow="18260" yWindow="-21100" windowWidth="38400" windowHeight="21100" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
added readme file, updated GACPAQ pages
</commit_message>
<xml_diff>
--- a/GACPAQ pages.xlsx
+++ b/GACPAQ pages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doncastillo/Code/gacpaq/gacpaq-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC74EE7C-8643-E448-9E10-69FBF77E6FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B78506-DD8D-A14D-901A-1884CBCBA742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18060" yWindow="-20240" windowWidth="38400" windowHeight="21100" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
+    <workbookView xWindow="-20140" yWindow="-21100" windowWidth="19200" windowHeight="19620" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="423">
   <si>
     <t>Page Number</t>
   </si>
@@ -3312,7 +3312,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3503,6 +3503,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8249,8 +8252,8 @@
       <c r="I9" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="J9" s="56" t="s">
-        <v>419</v>
+      <c r="J9" s="53" t="s">
+        <v>343</v>
       </c>
       <c r="K9" s="54" t="s">
         <v>422</v>
@@ -8298,8 +8301,8 @@
       <c r="F10" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="G10" s="53" t="s">
-        <v>337</v>
+      <c r="G10" s="56" t="s">
+        <v>415</v>
       </c>
       <c r="H10" s="53" t="s">
         <v>337</v>
@@ -8310,9 +8313,7 @@
       <c r="J10" s="56" t="s">
         <v>419</v>
       </c>
-      <c r="K10" s="54" t="s">
-        <v>422</v>
-      </c>
+      <c r="K10" s="80"/>
       <c r="L10" s="40" t="s">
         <v>281</v>
       </c>
@@ -8353,11 +8354,11 @@
       <c r="E11" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="F11" s="57" t="s">
-        <v>344</v>
-      </c>
-      <c r="G11" s="56" t="s">
-        <v>415</v>
+      <c r="F11" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="G11" s="53" t="s">
+        <v>337</v>
       </c>
       <c r="H11" s="53" t="s">
         <v>337</v>
@@ -8365,8 +8366,8 @@
       <c r="I11" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="J11" s="56" t="s">
-        <v>419</v>
+      <c r="J11" s="53" t="s">
+        <v>343</v>
       </c>
       <c r="K11" s="54" t="s">
         <v>422</v>

</xml_diff>

<commit_message>
enabled es-CL and hi-IN
</commit_message>
<xml_diff>
--- a/GACPAQ pages.xlsx
+++ b/GACPAQ pages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doncastillo/Code/gacpaq/gacpaq-app/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doncastillo/Code/gacpaq/gac-paq-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B78506-DD8D-A14D-901A-1884CBCBA742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DB6051E-5E4E-194A-A574-BADF491ACEBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20140" yWindow="-21100" windowWidth="19200" windowHeight="19620" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
+    <workbookView xWindow="18260" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="423">
   <si>
     <t>Page Number</t>
   </si>
@@ -2861,9 +2861,6 @@
     <t>Respostas enviadas</t>
   </si>
   <si>
-    <t>on-going</t>
-  </si>
-  <si>
     <t>India - English</t>
   </si>
   <si>
@@ -2884,6 +2881,9 @@
   </si>
   <si>
     <t>on-going (13)</t>
+  </si>
+  <si>
+    <t>on-going (14)</t>
   </si>
 </sst>
 </file>
@@ -3312,7 +3312,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3503,9 +3503,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5345,7 +5342,7 @@
       </c>
       <c r="E40" s="31"/>
       <c r="F40" s="32" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="G40" s="32"/>
       <c r="H40" s="31" t="s">
@@ -8013,8 +8010,8 @@
       <c r="F5" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="G5" s="56" t="s">
-        <v>415</v>
+      <c r="G5" s="53" t="s">
+        <v>337</v>
       </c>
       <c r="H5" s="53" t="s">
         <v>337</v>
@@ -8022,10 +8019,12 @@
       <c r="I5" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="J5" s="56" t="s">
-        <v>419</v>
-      </c>
-      <c r="K5" s="55"/>
+      <c r="J5" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="K5" s="54" t="s">
+        <v>422</v>
+      </c>
       <c r="L5" s="40" t="s">
         <v>335</v>
       </c>
@@ -8198,7 +8197,7 @@
         <v>343</v>
       </c>
       <c r="K8" s="54" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="L8" s="40" t="s">
         <v>336</v>
@@ -8226,10 +8225,10 @@
     </row>
     <row r="9" spans="1:36" ht="27" customHeight="1">
       <c r="A9" s="40" t="s">
+        <v>415</v>
+      </c>
+      <c r="B9" s="41" t="s">
         <v>416</v>
-      </c>
-      <c r="B9" s="41" t="s">
-        <v>417</v>
       </c>
       <c r="C9" s="53" t="s">
         <v>337</v>
@@ -8256,10 +8255,10 @@
         <v>343</v>
       </c>
       <c r="K9" s="54" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="L9" s="40" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="M9" s="48"/>
       <c r="N9" s="48"/>
@@ -8301,8 +8300,8 @@
       <c r="F10" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="G10" s="56" t="s">
-        <v>415</v>
+      <c r="G10" s="53" t="s">
+        <v>337</v>
       </c>
       <c r="H10" s="53" t="s">
         <v>337</v>
@@ -8310,10 +8309,12 @@
       <c r="I10" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="J10" s="56" t="s">
-        <v>419</v>
-      </c>
-      <c r="K10" s="80"/>
+      <c r="J10" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="K10" s="54" t="s">
+        <v>422</v>
+      </c>
       <c r="L10" s="40" t="s">
         <v>281</v>
       </c>
@@ -8370,7 +8371,7 @@
         <v>343</v>
       </c>
       <c r="K11" s="54" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="L11" s="40" t="s">
         <v>283</v>
@@ -8428,7 +8429,7 @@
         <v>343</v>
       </c>
       <c r="K12" s="54" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="L12" s="40" t="s">
         <v>285</v>
@@ -8486,7 +8487,7 @@
         <v>343</v>
       </c>
       <c r="K13" s="54" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="L13" s="40" t="s">
         <v>287</v>
@@ -8655,7 +8656,7 @@
         <v>337</v>
       </c>
       <c r="J16" s="56" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="K16" s="55"/>
       <c r="L16" s="40" t="s">
@@ -8709,7 +8710,7 @@
         <v>337</v>
       </c>
       <c r="J17" s="56" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="K17" s="55"/>
       <c r="L17" s="40" t="s">

</xml_diff>

<commit_message>
fixed height of the introductory section text container
</commit_message>
<xml_diff>
--- a/GACPAQ pages.xlsx
+++ b/GACPAQ pages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doncastillo/Code/gacpaq/gac-paq-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24EFBEE6-6C61-474D-B5F8-3918F106A171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{918DD141-9400-2547-9906-1BF85C017213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20140" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
+    <workbookView xWindow="18260" yWindow="-21000" windowWidth="38400" windowHeight="19220" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="425">
   <si>
     <t>Page Number</t>
   </si>
@@ -8239,10 +8239,18 @@
       <c r="B9" s="41" t="s">
         <v>424</v>
       </c>
-      <c r="C9" s="80"/>
-      <c r="D9" s="80"/>
-      <c r="E9" s="80"/>
-      <c r="F9" s="80"/>
+      <c r="C9" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="D9" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="E9" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="F9" s="53" t="s">
+        <v>337</v>
+      </c>
       <c r="G9" s="80"/>
       <c r="H9" s="80"/>
       <c r="I9" s="80"/>

</xml_diff>

<commit_message>
updated packages, added schema to the app.json
</commit_message>
<xml_diff>
--- a/GACPAQ pages.xlsx
+++ b/GACPAQ pages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doncastillo/Code/gacpaq/gac-paq-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{918DD141-9400-2547-9906-1BF85C017213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4CA96A-15E5-A241-90A2-BD5CC1540E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18260" yWindow="-21000" windowWidth="38400" windowHeight="19220" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
+    <workbookView xWindow="2720" yWindow="780" windowWidth="38400" windowHeight="19140" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3318,7 +3318,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3509,9 +3509,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8251,11 +8248,11 @@
       <c r="F9" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="G9" s="80"/>
-      <c r="H9" s="80"/>
-      <c r="I9" s="80"/>
-      <c r="J9" s="80"/>
-      <c r="K9" s="80"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
+      <c r="J9" s="55"/>
+      <c r="K9" s="55"/>
       <c r="L9" s="40" t="s">
         <v>423</v>
       </c>

</xml_diff>

<commit_message>
updated README file; added env and eas templates
</commit_message>
<xml_diff>
--- a/GACPAQ pages.xlsx
+++ b/GACPAQ pages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doncastillo/Code/gacpaq/gac-paq-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4CA96A-15E5-A241-90A2-BD5CC1540E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C598E79-F3CF-7743-8FFD-6518F40976E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2720" yWindow="780" windowWidth="38400" windowHeight="19140" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
+    <workbookView xWindow="-18660" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
enable main study for the en-GH
</commit_message>
<xml_diff>
--- a/GACPAQ pages.xlsx
+++ b/GACPAQ pages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doncastillo/Code/gacpaq/gac-paq-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C598E79-F3CF-7743-8FFD-6518F40976E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E57F109-8236-9C44-B350-5D7464212ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18660" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
+    <workbookView xWindow="18260" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="5" xr2:uid="{F0D6E043-EC2B-F746-8C39-25C7730C9E54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="985" uniqueCount="425">
   <si>
     <t>Page Number</t>
   </si>
@@ -8248,10 +8248,18 @@
       <c r="F9" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
-      <c r="J9" s="55"/>
+      <c r="G9" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="H9" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="I9" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="J9" s="53" t="s">
+        <v>337</v>
+      </c>
       <c r="K9" s="55"/>
       <c r="L9" s="40" t="s">
         <v>423</v>

</xml_diff>